<commit_message>
chore: refresh graded_slate 2026-04-02 after run_grader (fetch + regrade)
Regenerated from scripts/run_grader.ps1 -Date 2026-04-02; updates slate_eval,
ticket_eval_slate_latest.json, and committed graded workbooks for deploy.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/ui_runner/graded_slate/2026-04-02/graded_nba1h_2026-04-02.xlsx
+++ b/ui_runner/graded_slate/2026-04-02/graded_nba1h_2026-04-02.xlsx
@@ -691,7 +691,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>NBA SLATE GRADE  |  2026-04-02  |  Generated 2026-04-03 15:43</t>
+          <t>NBA SLATE GRADE  |  2026-04-02  |  Generated 2026-04-03 19:03</t>
         </is>
       </c>
     </row>
@@ -12259,7 +12259,7 @@
         <v>0.5558999999999999</v>
       </c>
       <c r="T100" s="8" t="n">
-        <v/>
+        <v>2</v>
       </c>
       <c r="U100" s="31" t="inlineStr">
         <is>
@@ -12924,7 +12924,7 @@
         <v>0.5451</v>
       </c>
       <c r="T107" s="4" t="n">
-        <v/>
+        <v>19</v>
       </c>
       <c r="U107" s="31" t="inlineStr">
         <is>
@@ -14159,7 +14159,7 @@
         <v>0.537</v>
       </c>
       <c r="T120" s="8" t="n">
-        <v/>
+        <v>10</v>
       </c>
       <c r="U120" s="31" t="inlineStr">
         <is>
@@ -15774,7 +15774,7 @@
         <v>0.5222</v>
       </c>
       <c r="T137" s="4" t="n">
-        <v/>
+        <v>8</v>
       </c>
       <c r="U137" s="31" t="inlineStr">
         <is>
@@ -17484,7 +17484,7 @@
         <v>0.4953</v>
       </c>
       <c r="T155" s="4" t="n">
-        <v/>
+        <v>10</v>
       </c>
       <c r="U155" s="31" t="inlineStr">
         <is>

</xml_diff>